<commit_message>
added partner bug list
</commit_message>
<xml_diff>
--- a/Defect_Temp.xlsx
+++ b/Defect_Temp.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500"/>
+    <workbookView windowWidth="20490" windowHeight="7500" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="samcomf" sheetId="1" r:id="rId1"/>
+    <sheet name="partner(app)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="114">
   <si>
     <t>Sr.No</t>
   </si>
@@ -149,7 +150,7 @@
     <t>(Screenshots, logs, or links)</t>
   </si>
   <si>
-    <t>001</t>
+    <t>0001</t>
   </si>
   <si>
     <t>Historical data index filter not working</t>
@@ -202,7 +203,7 @@
 https://sam-co.atlassian.net/browse/SMF-1451</t>
   </si>
   <si>
-    <t>002</t>
+    <t>0002</t>
   </si>
   <si>
     <t xml:space="preserve">Start Date field is missing
@@ -249,7 +250,7 @@
     <t>https://sam-co.atlassian.net/browse/SMF-1466?atlOrigin=eyJpIjoiZTNiMjgyMjYzY2ViNDY1ZThhZTBhMzdmZmRmMTI0ZjkiLCJwIjoiaiJ9</t>
   </si>
   <si>
-    <t>003</t>
+    <t>0003</t>
   </si>
   <si>
     <t>Validation Error</t>
@@ -279,7 +280,7 @@
     <t>Mannu Rajak</t>
   </si>
   <si>
-    <t>004</t>
+    <t>0004</t>
   </si>
   <si>
     <t>Maximum number of installment issue</t>
@@ -313,6 +314,118 @@
   <si>
     <t>Fahim Shaikh</t>
   </si>
+  <si>
+    <t>Investors Data missing in client summary</t>
+  </si>
+  <si>
+    <t>Client Summary section contain data of active and inactive investors when user check dashboard this investor data currently not there.</t>
+  </si>
+  <si>
+    <t>1.login to:-  https://dev-partners.samcomf.com/ 
+2.click on Dashboard icon.
+3.check count of active/inactive invesotor in client summary.</t>
+  </si>
+  <si>
+    <t>It must shows the data of active and inactive investors in client summary</t>
+  </si>
+  <si>
+    <t>There is no data in client summary.</t>
+  </si>
+  <si>
+    <t>18/07/2025</t>
+  </si>
+  <si>
+    <t>Partner(app)</t>
+  </si>
+  <si>
+    <t>Pratik</t>
+  </si>
+  <si>
+    <t>https://dev-partners.samcomf.com/distributor-dashboard</t>
+  </si>
+  <si>
+    <t>Folio number missing in Upcoming SIP’s section</t>
+  </si>
+  <si>
+    <t>Upcoming SIP’s section have data of investors uocoming sip details in that folio number is missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.login to:-  https://dev-partners.samcomf.com/ 
+2.click on Dashboard icon.
+3.click on Upcoming SIP’s section </t>
+  </si>
+  <si>
+    <t>Folio number must be there with invesor name.</t>
+  </si>
+  <si>
+    <t>Folio number missing</t>
+  </si>
+  <si>
+    <t>transaction amount is missing in cart list.</t>
+  </si>
+  <si>
+    <t>Cart list have transaction details like SIP,Lumpsum in that transaction amount is not there.</t>
+  </si>
+  <si>
+    <t>1.login to:-  https://dev-partners.samcomf.com/ 
+2.click on Transactions icon.
+3.click on cart list.
+4.click on any transaction.</t>
+  </si>
+  <si>
+    <t>transaction amount not there in cart list.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount is missing in cart list </t>
+  </si>
+  <si>
+    <t>https://dev-partners.samcomf.com/cart-list</t>
+  </si>
+  <si>
+    <t>Inaccurate SIP frequency type in mobile app</t>
+  </si>
+  <si>
+    <t>Instead of 'weekly' frequency there is 'Once a month' in mobile app.</t>
+  </si>
+  <si>
+    <t>Weekly' frequency SIP should be there.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 'Once a month' frequency type is there </t>
+  </si>
+  <si>
+    <t>Data is missing in downloaded Csv file</t>
+  </si>
+  <si>
+    <t>When user download csv file of 'smart transaction link' ;data is not there in csv file.</t>
+  </si>
+  <si>
+    <t>1.login to:-  https://dev-partners.samcomf.com/ 
+2.click on profile image.
+3.click on smart transaction link 
+4.select EUIN(optional)
+5.select scheme
+6.click on bulk download option.
+7.open the downloaded file.</t>
+  </si>
+  <si>
+    <t>when user download file based on selected scheme or EUIN data must be there in file.</t>
+  </si>
+  <si>
+    <t>Edit bank detail button not working</t>
+  </si>
+  <si>
+    <t>user unable to edit bank details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.login to:-  https://dev-partners.samcomf.com/ 
+2.click on profile image.
+3.Clicks on profile.
+4.click on Bank details 'Bank change request'edit  option </t>
+  </si>
+  <si>
+    <t xml:space="preserve">allow user to change bank details. </t>
+  </si>
 </sst>
 </file>
 
@@ -323,8 +436,8 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="179" formatCode="h:mm\ AM/PM"/>
+    <numFmt numFmtId="178" formatCode="h:mm\ AM/PM"/>
+    <numFmt numFmtId="179" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -351,18 +464,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="8" tint="-0.25"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8" tint="-0.25"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -843,7 +956,7 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -973,7 +1086,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -983,8 +1096,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -992,7 +1105,19 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1004,19 +1129,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
@@ -1027,6 +1149,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" quotePrefix="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1301,13 +1426,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1713,34 +1831,34 @@
       <c r="S2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="T2" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" s="3" customFormat="1" spans="2:20">
-      <c r="B3" s="6"/>
-      <c r="T3" s="12"/>
+    <row r="3" s="9" customFormat="1" spans="2:20">
+      <c r="B3" s="10"/>
+      <c r="T3" s="15"/>
     </row>
     <row r="4" customFormat="1" ht="105" spans="1:20">
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="11" t="s">
         <v>45</v>
       </c>
       <c r="H4" t="s">
@@ -1755,7 +1873,7 @@
       <c r="K4" t="s">
         <v>49</v>
       </c>
-      <c r="L4" s="10" t="s">
+      <c r="L4" s="14" t="s">
         <v>50</v>
       </c>
       <c r="M4" t="s">
@@ -1770,8 +1888,8 @@
       <c r="P4" t="s">
         <v>54</v>
       </c>
-      <c r="Q4" s="13"/>
-      <c r="T4" s="7" t="s">
+      <c r="Q4" s="16"/>
+      <c r="T4" s="11" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1779,22 +1897,22 @@
       <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="11" t="s">
         <v>59</v>
       </c>
       <c r="F6" t="s">
         <v>60</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="12" t="s">
         <v>61</v>
       </c>
       <c r="H6" t="s">
@@ -1809,7 +1927,7 @@
       <c r="K6" t="s">
         <v>49</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="14">
         <v>45723</v>
       </c>
       <c r="M6" t="s">
@@ -1827,13 +1945,13 @@
       <c r="Q6" t="s">
         <v>49</v>
       </c>
-      <c r="R6" s="10">
+      <c r="R6" s="14">
         <v>45754</v>
       </c>
       <c r="S6" t="s">
         <v>66</v>
       </c>
-      <c r="T6" s="14" t="s">
+      <c r="T6" s="17" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1841,22 +1959,22 @@
       <c r="A8">
         <v>3</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="20" t="s">
         <v>68</v>
       </c>
       <c r="C8" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="11" t="s">
         <v>73</v>
       </c>
       <c r="H8" t="s">
@@ -1871,7 +1989,7 @@
       <c r="K8" t="s">
         <v>49</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8" s="14">
         <v>45723</v>
       </c>
       <c r="M8" t="s">
@@ -1889,13 +2007,13 @@
       <c r="Q8" t="s">
         <v>49</v>
       </c>
-      <c r="R8" s="10">
+      <c r="R8" s="14">
         <v>45754</v>
       </c>
       <c r="S8" t="s">
         <v>66</v>
       </c>
-      <c r="T8" s="14" t="s">
+      <c r="T8" s="17" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1903,22 +2021,22 @@
       <c r="A10">
         <v>4</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="11" t="s">
         <v>80</v>
       </c>
       <c r="H10" t="s">
@@ -1933,14 +2051,14 @@
       <c r="K10" t="s">
         <v>81</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="14">
         <v>45754</v>
       </c>
       <c r="N10" t="s">
         <v>63</v>
       </c>
       <c r="O10" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="P10" t="s">
         <v>74</v>
@@ -1948,13 +2066,13 @@
       <c r="Q10" t="s">
         <v>81</v>
       </c>
-      <c r="R10" s="10">
+      <c r="R10" s="14">
         <v>45754</v>
       </c>
       <c r="S10" t="s">
         <v>66</v>
       </c>
-      <c r="T10" s="14" t="s">
+      <c r="T10" s="17" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1967,4 +2085,485 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="26.2857142857143" customWidth="1"/>
+    <col min="3" max="3" width="40.8571428571429" customWidth="1"/>
+    <col min="4" max="4" width="36.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="38" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="12.4285714285714" customWidth="1"/>
+    <col min="9" max="9" width="31" customWidth="1"/>
+    <col min="10" max="10" width="31.4285714285714" customWidth="1"/>
+    <col min="11" max="11" width="36.1428571428571" customWidth="1"/>
+    <col min="12" max="12" width="31.4285714285714" customWidth="1"/>
+    <col min="13" max="13" width="15.4285714285714" customWidth="1"/>
+    <col min="14" max="14" width="17.7142857142857" customWidth="1"/>
+    <col min="15" max="15" width="39.8571428571429" customWidth="1"/>
+    <col min="16" max="16" width="19" customWidth="1"/>
+    <col min="17" max="17" width="39.7142857142857" customWidth="1"/>
+    <col min="18" max="18" width="31.8571428571429" customWidth="1"/>
+    <col min="19" max="19" width="29.5714285714286" customWidth="1"/>
+    <col min="20" max="20" width="58.4285714285714" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" ht="17.25" spans="1:20">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" s="2" customFormat="1" spans="1:20">
+      <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T2" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" s="3" customFormat="1" ht="75" spans="1:20">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1001</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" s="3" customFormat="1" ht="60" spans="1:20">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1002</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="T4" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" s="3" customFormat="1" ht="75" spans="1:20">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1003</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" s="3" customFormat="1" ht="75" spans="1:20">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1004</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" s="3" customFormat="1" ht="120" spans="1:20">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3">
+        <v>1005</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="T7" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" s="3" customFormat="1" ht="90" spans="1:16">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1006</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" s="3" customFormat="1"/>
+    <row r="10" s="3" customFormat="1"/>
+    <row r="11" s="3" customFormat="1"/>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="T3" r:id="rId1" display="https://dev-partners.samcomf.com/distributor-dashboard"/>
+    <hyperlink ref="T4" r:id="rId1" display="https://dev-partners.samcomf.com/distributor-dashboard"/>
+    <hyperlink ref="T7" r:id="rId1" display="https://dev-partners.samcomf.com/distributor-dashboard"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>